<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-06 Le pique-nique de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-06.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-06.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison, jour de pluie</t>
+          <t>maison, jour de pluie, salon, panier, napperon, chaises, fenêtre, pain, fraises, poire, bol, corbeille</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, maman, papa</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La pluie annule le pique-nique du jardin. Nina dit qu'elle est déçue. Elles le font au salon. Plus tard, plus de fraises. Elle choisit une poire.</t>
+          <t>L'anse du panier pince le pouce de Nina. Sur le tissu, un éclat de napperon luit. Nina veut le pique-nique dehors, maintenant. La pluie mouille les chaises. Sourire parti. Envie et inquiétude dans la poitrine. Papa s'accroupit. Je suis déçue. Merci vécu. Pique-nique au salon. Deuxième ruse : plus de fraises, le bol glisse. Elle refuse de foncer. Une poire, alors. Un éclat de napperon tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière chante un air trop vite. L'eau y court, grise et claire. La fenêtre est toute embuée. Un doigt y a laissé une trace. Dehors, les chaises du jardin brillent. Elles sont mouillées, trop mouillées. Un panier attend sur le banc. La nappe dépasse, un peu froissée. Ça sent le pain, même d'ici. Tu as vu la gouttière, Nina ? Elle chante fort. C'est la pluie qui court. Tu veux dessiner sur la vitre ? Un petit soleil. Nina trace un rond dans la buée. En ce moment, Nina veut le jardin. On pique-nique dehors ? Regarde les chaises. Elles sont trop mouillées. Nina sent ses épaules tomber. Sa gorge se serre. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Nina souffle une fois. Sa buée s'ajoute à la vitre. Un pique-nique dans le salon ? Une autre idée. Bravo, Nina. J'apporte le panier. Elles posent la nappe au sol. Le tissu est à petits carreaux. Le pain sent le chaud. Tu veux une croûte ? Oui, maman. Papa pose deux tasses. Les tasses font un petit bruit. On est bien, ici. Presque comme dehors. Plus tard, Nina cherche les fraises. Des fraises ? Je regarde le bol. Le bol est vide. Il n'y en a plus. Nina sent encore sa gorge. Je suis déçue. Encore un souhait qui attend. Une autre idée ? Nina regarde la corbeille. Une poire, alors. Oui. Tu as proposé autre chose. Papa coupe la poire. Le cœur est doux et pâle. Nina croque. C'est juteux. Être déçue n'est pas honteux. Une autre idée peut venir. La pluie tapote encore, plus douce. La nappe reste au milieu du salon.</t>
+          <t>L'anse du panier pince le pouce de Nina. Aïe, ça pince, papa. Tu la vois, l'anse ? Oui, papa. Papa écarte l'anse, près du panier. Mes doigts bougent. Ils sont libres, Nina ? Oui, maman. Le panier sent le pain, même fermé. Ça sent le pain. Tu le sens, le pain chaud ? Oui, papa. Maman déplie un napperon, au bord du panier. Il est blanc, maman. Tu le vois, le napperon ? Oui, un peu froissé. Sur le tissu, un éclat de napperon luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Dehors, les chaises du jardin brillent, trop mouillées. Elles sont mouillées. Tu les vois, les chaises ? Oui, maman. La pluie tape sur la fenêtre, sans s'arrêter. Elle chante fort. C'est la pluie qui court. Sur le jardin. Nina pose le nez contre la fenêtre. Je veux le jardin. Tes pieds sont prêts, Nina ? Oui, maman. En ce moment, Nina veut le pique-nique dehors. On pique-nique dehors ? Tout de suite ? Oui, papa. Nina avance trop vite vers la porte. Sa main pousse la poignée. On y va ! Un filet d'eau glisse sous la porte. Il n'y a plus de jardin sec. Les chaises, Nina ? Trop mouillées. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tes épaules sont lourdes, Nina ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Nina ? Un peu, maman. Je suis déçue. L'éclat de napperon tremble, puis tient. Tu vois les chaises mouillées ? Oui. Nina serre les poings, puis les ouvre. Tes poings, Nina ? Ils se desserrent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière chante un air trop vite. L'eau y court, grise et claire. La fenêtre est toute embuée. Un doigt y a laissé une trace. Dehors, les chaises du jardin brillent. Elles sont mouillées, trop mouillées. Un panier attend sur le banc. La nappe dépasse, un peu froissée. Ça sent le pain, même d'ici. Tu as vu la gouttière, Nina ? Elle chante fort. C'est la pluie qui court. Tu veux dessiner sur la vitre ? Un petit soleil. Nina trace un rond dans la buée. En ce moment, Nina veut le jardin. On pique-nique dehors ? Regarde les chaises. Elles sont trop mouillées. Nina sent ses épaules tomber. Sa gorge se serre. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Nina souffle une fois. Sa buée s'ajoute à la vitre. Un pique-nique dans le salon ? Une autre idée. Bravo, Nina. J'apporte le panier. Elles posent la nappe au sol. Le tissu est à petits carreaux. Le pain sent le chaud. Tu veux une croûte ? Oui, maman. Papa pose deux tasses. Les tasses font un petit bruit. On est bien, ici. Presque comme dehors. Plus tard, Nina cherche les fraises. Des fraises ? Je regarde le bol. Le bol est vide. Il n'y en a plus. Nina sent encore sa gorge. Je suis déçue. Encore un souhait qui attend. Une autre idée ? Nina regarde la corbeille. Une poire, alors. Oui. Tu as proposé autre chose. Papa coupe la poire. Le cœur est doux et pâle. Nina croque. C'est juteux. Être déçue n'est pas honteux. Une autre idée peut venir. La pluie tapote encore, plus douce. La nappe reste au milieu du salon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'anse du panier pince le pouce de Nina. Aïe, ça pince, papa. Tu la vois, l'anse ? Oui, papa. Papa écarte l'anse, près du panier. Mes doigts bougent. Ils sont libres, Nina ? Oui, maman. Le panier sent le pain, même fermé. Ça sent le pain. Tu le sens, le pain chaud ? Oui, papa. Maman déplie un napperon, au bord du panier. Il est blanc, maman. Tu le vois, le napperon ? Oui, un peu froissé. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de napperon&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Dehors, les chaises du jardin brillent, trop mouillées. Elles sont mouillées. Tu les vois, les chaises ? Oui, maman. La pluie tape sur la fenêtre, sans s'arrêter. Elle chante fort. C'est la pluie qui court. Sur le jardin. Nina pose le nez contre la fenêtre. Je veux le jardin. Tes pieds sont prêts, Nina ? Oui, maman. En ce moment, Nina veut le pique-nique dehors. On pique-nique dehors ? Tout de suite ? Oui, papa. Nina avance trop vite vers la porte. Sa main pousse la poignée. On y va ! Un filet d'eau glisse sous la porte. Il n'y a plus de jardin sec. Les chaises, Nina ? Trop mouillées. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tes épaules sont lourdes, Nina ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Nina ? Un peu, maman. Je suis déçue. L'éclat de napperon tremble, puis tient. Tu vois les chaises mouillées ? Oui. Nina serre les poings, puis les ouvre. Tes poings, Nina ? Ils se desserrent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Fanny veut un pique-nique au jardin. La pluie tape sur la vitre. Fanny sent ses épaules tomber. Sa gorge se serre. Fanny dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Maman s'accroupit. Maman dit : un souhait peut attendre. On peut chercher une autre idée. Fanny souffle. Elle dit : un pique-nique dans le salon. Maman sourit. Elles posent une nappe. Le pain sent le chaud. Plus tard, Fanny veut des fraises. Il n'y en a plus. Fanny sent encore sa gorge. Elle dit : je suis déçue. Puis elle cherche une autre idée. Elle dit : une poire, alors. Papa coupe la poire. Être déçu n'est pas honteux. Une autre idée peut venir. [pause]</t>
+          <t>L'anse du panier pince le pouce de Nina. Aïe, ça pince, papa. Tu la vois, l'anse ? Oui, papa. Papa écarte l'anse, près du panier. Mes doigts bougent. Ils sont libres, Nina ? Oui, maman. Le panier sent le pain, même fermé. Ça sent le pain. Tu le sens, le pain chaud ? Oui, papa. Maman déplie un napperon, au bord du panier. Il est blanc, maman. Tu le vois, le napperon ? Oui, un peu froissé. Sur le tissu, un &lt;emphasis&gt;éclat de napperon&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Dehors, les chaises du jardin brillent, trop mouillées. Elles sont mouillées. Tu les vois, les chaises ? Oui, maman. La pluie tape sur la fenêtre, sans s'arrêter. Elle chante fort. C'est la pluie qui court. Sur le jardin. Nina pose le nez contre la fenêtre. Je veux le jardin. Tes pieds sont prêts, Nina ? Oui, maman. En ce moment, Nina veut le pique-nique dehors. On pique-nique dehors ? Tout de suite ? Oui, papa. Nina avance trop vite vers la porte. Sa main pousse la poignée. On y va ! Un filet d'eau glisse sous la porte. Il n'y a plus de jardin sec. Les chaises, Nina ? Trop mouillées. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Tes épaules sont lourdes, Nina ? Oui, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Nina ? Un peu, maman. Je suis déçue. L'éclat de napperon tremble, puis tient. Tu vois les chaises mouillées ? Oui. Nina serre les poings, puis les ouvre. Tes poings, Nina ? Ils se desserrent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de napperon</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,71 +1321,72 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_pique_nique_dehors_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La gouttière chante un air trop vite.
-narrateur|L'eau y court, grise et claire.
-narrateur|La fenêtre est toute embuée.
-narrateur|Un doigt y a laissé une trace.
-narrateur|Dehors, les chaises du jardin brillent.
-narrateur|Elles sont mouillées, trop mouillées.
-narrateur|Un panier attend sur le banc.
-narrateur|La nappe dépasse, un peu froissée.
-narrateur|Ça sent le pain, même d'ici.
-maman|Tu as vu la gouttière, Nina ?
+          <t>narrateur|L'anse du panier pince le pouce de Nina.
+enfant-f|Aïe, ça pince, papa.
+papa|Tu la vois, l'anse ?
+enfant-f|Oui, papa.
+narrateur|Papa écarte l'anse, près du panier.
+enfant-f|Mes doigts bougent.
+maman|Ils sont libres, Nina ?
+enfant-f|Oui, maman.
+narrateur|Le panier sent le pain, même fermé.
+enfant-f|Ça sent le pain.
+papa|Tu le sens, le pain chaud ?
+enfant-f|Oui, papa.
+narrateur|Maman déplie un napperon, au bord du panier.
+enfant-f|Il est blanc, maman.
+maman|Tu le vois, le napperon ?
+enfant-f|Oui, un peu froissé.
+narrateur|Sur le tissu, un éclat de napperon luit.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un point clair.
+narrateur|Dehors, les chaises du jardin brillent, trop mouillées.
+enfant-f|Elles sont mouillées.
+maman|Tu les vois, les chaises ?
+enfant-f|Oui, maman.
+narrateur|La pluie tape sur la fenêtre, sans s'arrêter.
 enfant-f|Elle chante fort.
 papa|C'est la pluie qui court.
-maman|Tu veux dessiner sur la vitre ?
-enfant-f|Un petit soleil.
-narrateur|Nina trace un rond dans la buée.
-narrateur|En ce moment, Nina veut le jardin.
+enfant-f|Sur le jardin.
+narrateur|Nina pose le nez contre la fenêtre.
+enfant-f|Je veux le jardin.
+maman|Tes pieds sont prêts, Nina ?
+enfant-f|Oui, maman.
+narrateur|En ce moment, Nina veut le pique-nique dehors.
 enfant-f|On pique-nique dehors ?
-maman|Regarde les chaises.
-maman|Elles sont trop mouillées.
-narrateur|Nina sent ses épaules tomber.
-narrateur|Sa gorge se serre.
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Nina avance trop vite vers la porte.
+narrateur|Sa main pousse la poignée.
+enfant-f|On y va !
+narrateur|Un filet d'eau glisse sous la porte.
+enfant-f|Il n'y a plus de jardin sec.
+maman|Les chaises, Nina ?
+enfant-f|Trop mouillées.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+enfant-f|J'ai mal au ventre.
+papa|Tes épaules sont lourdes, Nina ?
+enfant-f|Oui, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Nina ?
+enfant-f|Un peu, maman.
 enfant-f|Je suis déçue.
-maman|Tu es déçue.
-maman|Ce n'est pas honteux.
-maman|Un souhait peut attendre.
-maman|On peut chercher une autre idée.
-narrateur|Nina souffle une fois.
-narrateur|Sa buée s'ajoute à la vitre.
-enfant-f|Un pique-nique dans le salon ?
-maman|Une autre idée.
-maman|Bravo, Nina.
-papa|J'apporte le panier.
-narrateur|Elles posent la nappe au sol.
-narrateur|Le tissu est à petits carreaux.
-narrateur|Le pain sent le chaud.
-maman|Tu veux une croûte ?
-enfant-f|Oui, maman.
-narrateur|Papa pose deux tasses.
-narrateur|Les tasses font un petit bruit.
-papa|On est bien, ici.
-enfant-f|Presque comme dehors.
-narrateur|Plus tard, Nina cherche les fraises.
-enfant-f|Des fraises ?
-papa|Je regarde le bol.
-narrateur|Le bol est vide.
-papa|Il n'y en a plus.
-narrateur|Nina sent encore sa gorge.
-enfant-f|Je suis déçue.
-papa|Encore un souhait qui attend.
-maman|Une autre idée ?
-narrateur|Nina regarde la corbeille.
-enfant-f|Une poire, alors.
-papa|Oui.
-maman|Tu as proposé autre chose.
-narrateur|Papa coupe la poire.
-narrateur|Le cœur est doux et pâle.
-narrateur|Nina croque.
-enfant-f|C'est juteux.
-maman|Être déçue n'est pas honteux.
-papa|Une autre idée peut venir.
-narrateur|La pluie tapote encore, plus douce.
-narrateur|La nappe reste au milieu du salon.</t>
+narrateur|L'éclat de napperon tremble, puis tient.
+papa|Tu vois les chaises mouillées ?
+enfant-f|Oui.
+narrateur|Nina serre les poings, puis les ouvre.
+papa|Tes poings, Nina ?
+enfant-f|Ils se desserrent.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1422,12 +1423,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>La pluie arrive. Que dit Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La pluie arrive. Que dit &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>La pluie arrive. Que dit Fanny ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;La pluie arrive. Que dit &lt;emphasis&gt;Nina&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1452,7 +1453,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Fanny cherche une autre idée. Que dit-elle d'abord ?</t>
+          <t>Nina cherche une autre idée. Que dit-elle d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1490,18 +1491,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1516,34 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1552,23 +1557,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_pluie_arrive_que_dit_nina; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1601,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a encore un bout de poire. J'ai dit : je suis déçue. Oui. Le souhait peut attendre. Une autre idée est arrivée. Le salon, puis la poire. Bravo, Nina. Deux autres idées. Oui. Une goutte court encore sur la vitre.</t>
+          <t>Nina avance trop vite vers le panier. Je prends tout, maintenant ! Les mots se bousculent dans sa bouche. Le jardin, dehors. Nina avance les mains, trop vite. Puis elle s'arrête. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le napperon, un instant. Elle écoute la pluie, près de la fenêtre. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le napperon est froid, sous les doigts. Il est lisse. Un pique-nique dans le salon ? Tu le vois, le salon ? Oui, maman. On pose le napperon au sol ? Oui, papa. Ils déplient le napperon, sans se presser. Le tissu sent le pain, un peu. Ça sent le pain. Tu veux une croûte ? Oui, maman. Papa pose deux tasses, tout petit. Les tasses font un petit bruit. On est bien, ici. Presque comme dehors. Le ventre de Nina se desserre. Les épaules se relèvent un peu. Tes joues sont chaudes, Nina ? Un peu, maman. Le pain est chaud, Nina ? Oui, papa. Le coin du napperon tient, au salon. On est là.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a encore un bout de poire. J'ai dit : je suis déçue. Oui. Le souhait peut attendre. Une autre idée est arrivée. Le salon, puis la poire. Bravo, Nina. Deux autres idées. Oui. Une goutte court encore sur la vitre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina avance trop vite vers le panier. Je prends tout, maintenant ! Les mots se bousculent dans sa bouche. Le jardin, dehors. Nina avance les mains, trop vite. Puis elle s'arrête. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le napperon, un instant. Elle écoute la pluie, près de la fenêtre. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le napperon est froid, sous les doigts. Il est lisse. Un pique-nique dans le &lt;emphasis level="moderate"&gt;salon&lt;/emphasis&gt; ? Tu le vois, le salon ? Oui, maman. On pose le napperon au sol ? Oui, papa. Ils déplient le napperon, sans se presser. Le tissu sent le pain, un peu. Ça sent le pain. Tu veux une croûte ? Oui, maman. Papa pose deux tasses, tout petit. Les tasses font un petit bruit. On est bien, ici. Presque comme dehors. Le ventre de Nina se desserre. Les épaules se relèvent un peu. Tes joues sont chaudes, Nina ? Un peu, maman. Le pain est chaud, Nina ? Oui, papa. Le coin du napperon tient, au salon. On est là.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Fanny a nommé : &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Le souhait peut attendre. Une autre idée est arrivée. Papa et maman étaient là. [pause]</t>
+          <t>Nina avance trop vite vers le panier. Je prends tout, maintenant ! Les mots se bousculent dans sa bouche. Le jardin, dehors. Nina avance les mains, trop vite. Puis elle s'arrête. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le napperon, un instant. Elle écoute la pluie, près de la fenêtre. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le napperon est froid, sous les doigts. Il est lisse. Un pique-nique dans le &lt;emphasis&gt;salon&lt;/emphasis&gt; ? Tu le vois, le salon ? Oui, maman. On pose le napperon au sol ? Oui, papa. Ils déplient le napperon, sans se presser. Le tissu sent le pain, un peu. Ça sent le pain. Tu veux une croûte ? Oui, maman. Papa pose deux tasses, tout petit. Les tasses font un petit bruit. On est bien, ici. Presque comme dehors. Le ventre de Nina se desserre. Les épaules se relèvent un peu. Tes joues sont chaudes, Nina ? Un peu, maman. Le pain est chaud, Nina ? Oui, papa. Le coin du napperon tient, au salon. On est là. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1658,7 +1663,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1666,10 +1671,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1692,30 +1697,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>salon</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1724,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1740,21 +1745,50 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=elle_propose_le_salon_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a encore un bout de poire.
-enfant-f|J'ai dit : je suis déçue.
-maman|Oui.
-maman|Le souhait peut attendre.
-papa|Une autre idée est arrivée.
-maman|Le salon, puis la poire.
-maman|Bravo, Nina.
-enfant-f|Deux autres idées.
-maman|Oui.
-narrateur|Une goutte court encore sur la vitre.</t>
+          <t>narrateur|Nina avance trop vite vers le panier.
+enfant-f|Je prends tout, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Le jardin, dehors.
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le napperon, un instant.
+narrateur|Elle écoute la pluie, près de la fenêtre.
+papa|Tu restes un peu, Nina ?
+enfant-f|Oui, papa.
+papa|Merci, Nina.
+narrateur|Papa reste à la même hauteur.
+maman|Le napperon est froid, sous les doigts.
+enfant-f|Il est lisse.
+enfant-f|Un pique-nique dans le salon ?
+maman|Tu le vois, le salon ?
+enfant-f|Oui, maman.
+papa|On pose le napperon au sol ?
+enfant-f|Oui, papa.
+narrateur|Ils déplient le napperon, sans se presser.
+narrateur|Le tissu sent le pain, un peu.
+enfant-f|Ça sent le pain.
+maman|Tu veux une croûte ?
+enfant-f|Oui, maman.
+narrateur|Papa pose deux tasses, tout petit.
+narrateur|Les tasses font un petit bruit.
+papa|On est bien, ici.
+enfant-f|Presque comme dehors.
+narrateur|Le ventre de Nina se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tes joues sont chaudes, Nina ?
+enfant-f|Un peu, maman.
+papa|Le pain est chaud, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le coin du napperon tient, au salon.
+enfant-f|On est là.</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1815,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina croque la poire. Maman plie un coin de la nappe. On reste assis un peu ? Oui, maman. Tu as nommé : déçue. Puis tu as cherché. Le pain sent encore le chaud. La gouttière chante plus lentement. Le salon, c'est bien aussi. Oui. Avec l'autre idée.</t>
+          <t>Nina cherche les fraises, trop vite. Des fraises, maintenant ! Le bol du panier tremble, presque vide. Il n'y en a plus. Les fraises, Nina ? Parti. Les épaules de Nina retombent. Je les prends, tout de suite ! Nina avance trop vite vers le bol. Le bol glisse au bord. Il part ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le napperon, un instant. Elle écoute le salon, près du pain. Sur le tissu, un éclat de napperon luit. Là, sur le tissu. Tu vois le point, Nina ? Oui, papa. Nina lève les yeux vers la corbeille. Une poire, alors. Tu la vois, la poire ? Oui, maman. Elle est jaune, Nina ? Un peu verte. Papa coupe la poire, sans se presser. Le cœur est doux et pâle. C'est juteux. La poire a failli glisser, un moment. Elle a failli partir. Elle tient, Nina ? Oui, papa. Nina croque, sans se bousculer. Tes doigts sont froids, Nina ? Un peu, maman. On reste près du napperon ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina croque la poire. Maman plie un coin de la nappe. On reste assis un peu ? Oui, maman. Tu as nommé : déçue. Puis tu as cherché. Le pain sent encore le chaud. La gouttière chante plus lentement. Le salon, c'est bien aussi. Oui. Avec l'autre idée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina cherche les fraises, trop vite. Des fraises, maintenant ! Le bol du panier tremble, presque vide. Il n'y en a plus. Les fraises, Nina ? Parti. Les épaules de Nina retombent. Je les prends, tout de suite ! Nina avance trop vite vers le bol. Le bol glisse au bord. Il part ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le napperon, un instant. Elle écoute le salon, près du pain. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de napperon&lt;/emphasis&gt; luit. Là, sur le tissu. Tu vois le point, Nina ? Oui, papa. Nina lève les yeux vers la corbeille. Une poire, alors. Tu la vois, la poire ? Oui, maman. Elle est jaune, Nina ? Un peu verte. Papa coupe la poire, sans se presser. Le cœur est doux et pâle. C'est juteux. La poire a failli glisser, un moment. Elle a failli partir. Elle tient, Nina ? Oui, papa. Nina croque, sans se bousculer. Tes doigts sont froids, Nina ? Un peu, maman. On reste près du napperon ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Fanny croque la poire. Maman plie la nappe. Ils s'assoient. [pause]</t>
+          <t>Nina cherche les fraises, trop vite. Des fraises, maintenant ! Le bol du panier tremble, presque vide. Il n'y en a plus. Les fraises, Nina ? Parti. Les épaules de Nina retombent. Je les prends, tout de suite ! Nina avance trop vite vers le bol. Le bol glisse au bord. Il part ! Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le napperon, un instant. Elle écoute le salon, près du pain. Sur le tissu, un &lt;emphasis&gt;éclat de napperon&lt;/emphasis&gt; luit. Là, sur le tissu. Tu vois le point, Nina ? Oui, papa. Nina lève les yeux vers la corbeille. Une poire, alors. Tu la vois, la poire ? Oui, maman. Elle est jaune, Nina ? Un peu verte. Papa coupe la poire, sans se presser. Le cœur est doux et pâle. C'est juteux. La poire a failli glisser, un moment. Elle a failli partir. Elle tient, Nina ? Oui, papa. Nina croque, sans se bousculer. Tes doigts sont froids, Nina ? Un peu, maman. On reste près du napperon ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1872,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,10 +1880,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1870,28 +1904,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de napperon</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1938,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1914,20 +1952,53 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=plus_de_fraises_elle_refuse_de_foncer_elle_propose_une_poire; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina croque la poire.
-narrateur|Maman plie un coin de la nappe.
-maman|On reste assis un peu ?
+          <t>narrateur|Nina cherche les fraises, trop vite.
+enfant-f|Des fraises, maintenant !
+narrateur|Le bol du panier tremble, presque vide.
+enfant-f|Il n'y en a plus.
+maman|Les fraises, Nina ?
+enfant-f|Parti.
+narrateur|Les épaules de Nina retombent.
+enfant-f|Je les prends, tout de suite !
+narrateur|Nina avance trop vite vers le bol.
+narrateur|Le bol glisse au bord.
+enfant-f|Il part !
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le napperon, un instant.
+narrateur|Elle écoute le salon, près du pain.
+narrateur|Sur le tissu, un éclat de napperon luit.
+enfant-f|Là, sur le tissu.
+papa|Tu vois le point, Nina ?
+enfant-f|Oui, papa.
+narrateur|Nina lève les yeux vers la corbeille.
+enfant-f|Une poire, alors.
+maman|Tu la vois, la poire ?
 enfant-f|Oui, maman.
-papa|Tu as nommé : déçue.
-papa|Puis tu as cherché.
-narrateur|Le pain sent encore le chaud.
-narrateur|La gouttière chante plus lentement.
-enfant-f|Le salon, c'est bien aussi.
-maman|Oui.
-maman|Avec l'autre idée.</t>
+papa|Elle est jaune, Nina ?
+enfant-f|Un peu verte.
+narrateur|Papa coupe la poire, sans se presser.
+narrateur|Le cœur est doux et pâle.
+enfant-f|C'est juteux.
+narrateur|La poire a failli glisser, un moment.
+enfant-f|Elle a failli partir.
+papa|Elle tient, Nina ?
+enfant-f|Oui, papa.
+narrateur|Nina croque, sans se bousculer.
+maman|Tes doigts sont froids, Nina ?
+enfant-f|Un peu, maman.
+papa|On reste près du napperon ?
+enfant-f|Oui.</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2025,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Nina. La nappe reste un moment par terre.</t>
+          <t>Ils restent près du napperon. Maman plie un coin du tissu. La poire a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Nina tapote le tissu du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La poire est restée, Nina. Oui, avec nous. Ça sent le pain, un peu tiède. Et le tissu, maman. Oui, dans l'air. La pluie tape plus lentement, Nina ? Oui, papa. Le napperon reste au milieu du salon. Un éclat de napperon tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Nina. La nappe reste un moment par terre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du napperon. Maman plie un coin du tissu. La poire a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Nina tapote le tissu du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La poire est restée, Nina. Oui, avec nous. Ça sent le pain, un peu tiède. Et le tissu, maman. Oui, dans l'air. La pluie tape plus lentement, Nina ? Oui, papa. Le napperon reste au milieu du salon. Un &lt;emphasis level="moderate"&gt;éclat de napperon&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du napperon. Maman plie un coin du tissu. La poire a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Nina tapote le tissu du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La poire est restée, Nina. Oui, avec nous. Ça sent le pain, un peu tiède. Et le tissu, maman. Oui, dans l'air. La pluie tape plus lentement, Nina ? Oui, papa. Le napperon reste au milieu du salon. Un &lt;emphasis&gt;éclat de napperon&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2082,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2102,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2116,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de napperon</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2139,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,27 +2152,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis déçue.
-enfant-f|J'ai trouvé une autre idée.
-maman|Bravo, Nina.
-narrateur|La nappe reste un moment par terre.</t>
+          <t>narrateur|Ils restent près du napperon.
+narrateur|Maman plie un coin du tissu.
+enfant-f|La poire a une trace, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, près du bord.
+maman|On est bien, ici.
+narrateur|Nina tapote le tissu du doigt.
+enfant-f|Il a une trace de jus.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|La poire est restée, Nina.
+enfant-f|Oui, avec nous.
+narrateur|Ça sent le pain, un peu tiède.
+enfant-f|Et le tissu, maman.
+maman|Oui, dans l'air.
+papa|La pluie tape plus lentement, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le napperon reste au milieu du salon.
+narrateur|Un éclat de napperon tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2168,6 +2262,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>